<commit_message>
Updated high low motif files. In addition, updated Dataframes_with_features, Selected_features and xgb_best_params files only to add easily eyals code to the pipeline, before running everything on mac\linux
</commit_message>
<xml_diff>
--- a/xgb_RNAp_best_params.xlsx
+++ b/xgb_RNAp_best_params.xlsx
@@ -467,71 +467,71 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2042648709315376</v>
+        <v>0.5437977660199882</v>
       </c>
       <c r="B2" t="n">
-        <v>288</v>
+        <v>3825</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05532058682058681</v>
+        <v>0.1357048465023773</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7206990540323873</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0001459420780408435</v>
+        <v>0.4749420675346601</v>
       </c>
       <c r="G2" t="n">
-        <v>0.194389624932033</v>
+        <v>0.9127633992796768</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.8383838383838383</v>
       </c>
       <c r="B3" t="n">
-        <v>288</v>
+        <v>453</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>0.06667333333333332</v>
+        <v>0.3092404558404557</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.5688572972523589</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0001222222222222222</v>
+        <v>0.9037999037999038</v>
       </c>
       <c r="G3" t="n">
-        <v>0.09454377456600671</v>
+        <v>0.9122316941477339</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.7142857142857143</v>
+        <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>618</v>
+        <v>3666</v>
       </c>
       <c r="C4" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01852592592592592</v>
+        <v>0.2037851851851851</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.368431580575495</v>
+        <v>0.9115283680764379</v>
       </c>
     </row>
     <row r="5">
@@ -539,22 +539,22 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>3333</v>
+        <v>285</v>
       </c>
       <c r="C5" t="n">
         <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>0.240837037037037</v>
+        <v>0.034405291005291</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0.417283950617284</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3333333333333334</v>
+        <v>0.7779333333333334</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2435663366001412</v>
+        <v>0.9207549390425377</v>
       </c>
     </row>
     <row r="6">
@@ -562,22 +562,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>3000</v>
+        <v>3666</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3333666666666666</v>
+        <v>0.2778888888888889</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>0.495</v>
+        <v>0.6667</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.02330854112447889</v>
+        <v>0.9108917116349641</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix missing scale step before predictionin main, and update the scale function in model functions
</commit_message>
<xml_diff>
--- a/xgb_RNAp_best_params.xlsx
+++ b/xgb_RNAp_best_params.xlsx
@@ -467,48 +467,48 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.5437977660199882</v>
+        <v>0.7083870252594533</v>
       </c>
       <c r="B2" t="n">
-        <v>3825</v>
+        <v>824</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1357048465023773</v>
+        <v>0.1270832159423837</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4749420675346601</v>
+        <v>0.7100967701708443</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9127633992796768</v>
+        <v>0.8853353640074517</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.8383838383838383</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="B3" t="n">
-        <v>453</v>
+        <v>333</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3092404558404557</v>
+        <v>0.05557777777777777</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5688572972523589</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9037999037999038</v>
+        <v>0.3334</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9122316941477339</v>
+        <v>0.8883196868105148</v>
       </c>
     </row>
     <row r="4">
@@ -516,22 +516,22 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>3666</v>
+        <v>333</v>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2037851851851851</v>
+        <v>0.05557777777777777</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0.2593111111111111</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9115283680764379</v>
+        <v>0.8981262094521473</v>
       </c>
     </row>
     <row r="5">
@@ -539,45 +539,45 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>285</v>
+        <v>778</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>0.034405291005291</v>
+        <v>0.2407481481481481</v>
       </c>
       <c r="E5" t="n">
-        <v>0.417283950617284</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7779333333333334</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9207549390425377</v>
+        <v>0.8752097823918568</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="B6" t="n">
-        <v>3666</v>
+        <v>333</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2778888888888889</v>
+        <v>0.05557777777777777</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.2592592592592593</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6667</v>
+        <v>0.7407444444444444</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9108917116349641</v>
+        <v>0.8927200059591917</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rn ai main combining (#30)
* Added RNAi to entire pipeline, added function to call RNAi or RNAp running from main, renamed RNAp files to start with RNAp_

* Updated before merging to main

---------

Co-authored-by: iGem <igem@davids-MacBook-Pro.local>
</commit_message>
<xml_diff>
--- a/xgb_RNAp_best_params.xlsx
+++ b/xgb_RNAp_best_params.xlsx
@@ -467,117 +467,117 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.7083870252594533</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="B2" t="n">
-        <v>824</v>
+        <v>1386</v>
       </c>
       <c r="C2" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1270832159423837</v>
+        <v>0.172026455026455</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7100967701708443</v>
+        <v>0.4172903703703704</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8853353640074517</v>
+        <v>0.8799143542907113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="B3" t="n">
-        <v>333</v>
+        <v>778</v>
       </c>
       <c r="C3" t="n">
         <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05557777777777777</v>
+        <v>0.1296814814814815</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3334</v>
+        <v>0.4814888888888889</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8883196868105148</v>
+        <v>0.8786891468194422</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="B4" t="n">
-        <v>333</v>
+        <v>1000</v>
       </c>
       <c r="C4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
         <v>0.05557777777777777</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2593111111111111</v>
+        <v>0.3334</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8981262094521473</v>
+        <v>0.885596187827569</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="B5" t="n">
-        <v>778</v>
+        <v>1223</v>
       </c>
       <c r="C5" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2407481481481481</v>
+        <v>0.1</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0.7407444444444444</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8752097823918568</v>
+        <v>0.8580939049640175</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.495</v>
       </c>
       <c r="B6" t="n">
-        <v>333</v>
+        <v>1000</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>0.05557777777777777</v>
+        <v>0.1667333333333333</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2592592592592593</v>
+        <v>0.4</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7407444444444444</v>
+        <v>0.495</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8927200059591917</v>
+        <v>0.8766384352011001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>